<commit_message>
chore(kb): align knowledge base with mandatory dual-input workflow
</commit_message>
<xml_diff>
--- a/knowledge_base/source/04_requirements.xlsx
+++ b/knowledge_base/source/04_requirements.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_requirements" sheetId="1" r:id="R096ad6b6969f4ba8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_requirements" sheetId="1" r:id="R194e9f36926941a0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -772,7 +772,7 @@
         <x:v>System Defined</x:v>
       </x:c>
       <x:c r="H11" s="16" t="str">
-        <x:v>All analyses</x:v>
+        <x:v>Entire analysis</x:v>
       </x:c>
       <x:c r="I11" s="16" t="str">
         <x:v>Deterministic validation</x:v>
@@ -810,7 +810,7 @@
         <x:v>Derived</x:v>
       </x:c>
       <x:c r="H12" s="16" t="str">
-        <x:v>Exam only</x:v>
+        <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I12" s="16" t="str">
         <x:v>Text-quality analysis</x:v>
@@ -848,7 +848,7 @@
         <x:v>Derived</x:v>
       </x:c>
       <x:c r="H13" s="16" t="str">
-        <x:v>Exam only</x:v>
+        <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I13" s="16" t="str">
         <x:v>Text-quality analysis</x:v>
@@ -886,7 +886,7 @@
         <x:v>Derived</x:v>
       </x:c>
       <x:c r="H14" s="16" t="str">
-        <x:v>Exam only</x:v>
+        <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I14" s="16" t="str">
         <x:v>Content-completeness analysis</x:v>
@@ -924,7 +924,7 @@
         <x:v>Derived</x:v>
       </x:c>
       <x:c r="H15" s="16" t="str">
-        <x:v>Exam only</x:v>
+        <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I15" s="16" t="str">
         <x:v>Document and layout validation</x:v>
@@ -962,7 +962,7 @@
         <x:v>Derived</x:v>
       </x:c>
       <x:c r="H16" s="16" t="str">
-        <x:v>Exam only</x:v>
+        <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I16" s="16" t="str">
         <x:v>Visual and OCR analysis</x:v>
@@ -1000,7 +1000,7 @@
         <x:v>Derived</x:v>
       </x:c>
       <x:c r="H17" s="16" t="str">
-        <x:v>Exam only</x:v>
+        <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I17" s="16" t="str">
         <x:v>Layout analysis</x:v>
@@ -1038,7 +1038,7 @@
         <x:v>Derived</x:v>
       </x:c>
       <x:c r="H18" s="16" t="str">
-        <x:v>Exam only</x:v>
+        <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I18" s="16" t="str">
         <x:v>Marks extraction</x:v>
@@ -1076,7 +1076,7 @@
         <x:v>Derived</x:v>
       </x:c>
       <x:c r="H19" s="16" t="str">
-        <x:v>Exam only</x:v>
+        <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I19" s="16" t="str">
         <x:v>Arithmetic validation</x:v>
@@ -1114,7 +1114,7 @@
         <x:v>Derived</x:v>
       </x:c>
       <x:c r="H20" s="16" t="str">
-        <x:v>Exam only</x:v>
+        <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I20" s="16" t="str">
         <x:v>Structural analysis</x:v>
@@ -1152,7 +1152,7 @@
         <x:v>Derived</x:v>
       </x:c>
       <x:c r="H21" s="16" t="str">
-        <x:v>Exam only</x:v>
+        <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I21" s="16" t="str">
         <x:v>Metadata extraction</x:v>
@@ -1190,7 +1190,7 @@
         <x:v>Derived</x:v>
       </x:c>
       <x:c r="H22" s="16" t="str">
-        <x:v>Exam only</x:v>
+        <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I22" s="16" t="str">
         <x:v>Instruction analysis</x:v>
@@ -1228,7 +1228,7 @@
         <x:v>Derived</x:v>
       </x:c>
       <x:c r="H23" s="16" t="str">
-        <x:v>Exam only</x:v>
+        <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I23" s="16" t="str">
         <x:v>Cross-reference and layout analysis</x:v>
@@ -1266,7 +1266,7 @@
         <x:v>System Defined</x:v>
       </x:c>
       <x:c r="H24" s="16" t="str">
-        <x:v>Exam only</x:v>
+        <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I24" s="16" t="str">
         <x:v>Input validation</x:v>
@@ -1304,7 +1304,7 @@
         <x:v>System Defined</x:v>
       </x:c>
       <x:c r="H25" s="16" t="str">
-        <x:v>TP-153</x:v>
+        <x:v>TP-153 evidence only</x:v>
       </x:c>
       <x:c r="I25" s="16" t="str">
         <x:v>Table validation</x:v>
@@ -1342,7 +1342,7 @@
         <x:v>System Defined</x:v>
       </x:c>
       <x:c r="H26" s="16" t="str">
-        <x:v>TP-153</x:v>
+        <x:v>TP-153 evidence only</x:v>
       </x:c>
       <x:c r="I26" s="16" t="str">
         <x:v>Table validation</x:v>
@@ -1371,7 +1371,7 @@
         <x:v>Usable Assessment Data</x:v>
       </x:c>
       <x:c r="E27" s="16" t="str">
-        <x:v>TP-153 assessment methods or activities should be readable when required for comparison.</x:v>
+        <x:v>TP-153 assessment methods or activities required for the analysis should be present, readable, and usable.</x:v>
       </x:c>
       <x:c r="F27" s="16" t="str">
         <x:v>System Requirement</x:v>
@@ -1380,7 +1380,7 @@
         <x:v>System Defined</x:v>
       </x:c>
       <x:c r="H27" s="16" t="str">
-        <x:v>TP-153</x:v>
+        <x:v>TP-153 evidence only</x:v>
       </x:c>
       <x:c r="I27" s="16" t="str">
         <x:v>Table validation</x:v>
@@ -1389,7 +1389,7 @@
         <x:v>Assessment section is missing or unreadable</x:v>
       </x:c>
       <x:c r="K27" s="16" t="str">
-        <x:v>Assessment comparison is not requested</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="L27" s="22" t="str">
         <x:v>Missing data results in Not Verified.</x:v>
@@ -1418,7 +1418,7 @@
         <x:v>System Defined</x:v>
       </x:c>
       <x:c r="H28" s="16" t="str">
-        <x:v>Generated report</x:v>
+        <x:v>Generated report output</x:v>
       </x:c>
       <x:c r="I28" s="16" t="str">
         <x:v>Report validation</x:v>
@@ -1456,7 +1456,7 @@
         <x:v>System Defined</x:v>
       </x:c>
       <x:c r="H29" s="16" t="str">
-        <x:v>Generated report</x:v>
+        <x:v>Generated report output</x:v>
       </x:c>
       <x:c r="I29" s="16" t="str">
         <x:v>Policy validation</x:v>
@@ -1494,7 +1494,7 @@
         <x:v>System Defined</x:v>
       </x:c>
       <x:c r="H30" s="16" t="str">
-        <x:v>All analyses</x:v>
+        <x:v>Entire analysis</x:v>
       </x:c>
       <x:c r="I30" s="16" t="str">
         <x:v>Deterministic validation</x:v>
@@ -1532,7 +1532,7 @@
         <x:v>System Defined</x:v>
       </x:c>
       <x:c r="H31" s="24" t="str">
-        <x:v>All analyses</x:v>
+        <x:v>Entire analysis</x:v>
       </x:c>
       <x:c r="I31" s="24" t="str">
         <x:v>Report validation</x:v>
@@ -1550,7 +1550,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27ea5a9d459341d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd5b2cd2d3b74564"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Prepare deployment and improve Arabic exam extraction
</commit_message>
<xml_diff>
--- a/knowledge_base/source/04_requirements.xlsx
+++ b/knowledge_base/source/04_requirements.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_requirements" sheetId="1" r:id="R194e9f36926941a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_requirements" sheetId="1" r:id="R556617bc92f44355"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -116,7 +116,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="26">
+  <x:cellXfs count="27">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -179,6 +179,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -801,7 +802,7 @@
         <x:v>Clear Task Statement</x:v>
       </x:c>
       <x:c r="E12" s="16" t="str">
-        <x:v>Each question should state a clear task and recognizable response expectation.</x:v>
+        <x:v>Each question should state a recognizable action and the response or output expected from the student.</x:v>
       </x:c>
       <x:c r="F12" s="16" t="str">
         <x:v>Derived Exam Requirement</x:v>
@@ -813,16 +814,16 @@
         <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I12" s="16" t="str">
-        <x:v>Text-quality analysis</x:v>
+        <x:v>Question-text task analysis</x:v>
       </x:c>
       <x:c r="J12" s="16" t="str">
-        <x:v>OCR confidence is insufficient</x:v>
+        <x:v>Question text is unreadable or OCR confidence is insufficient</x:v>
       </x:c>
       <x:c r="K12" s="16" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="L12" s="22" t="str">
-        <x:v>Style preferences alone are not evaluated.</x:v>
+        <x:v>Limited to the task action and expected response; supporting-material availability, information completeness, and exam-level instructions are evaluated separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
@@ -839,7 +840,7 @@
         <x:v>Unambiguous Wording</x:v>
       </x:c>
       <x:c r="E13" s="16" t="str">
-        <x:v>Question wording should avoid ambiguity, contradiction, or missing conditions that materially affect interpretation.</x:v>
+        <x:v>Question wording should avoid linguistic ambiguity, contradiction, unclear terminology, or wording that materially permits different interpretations.</x:v>
       </x:c>
       <x:c r="F13" s="16" t="str">
         <x:v>Derived Exam Requirement</x:v>
@@ -851,16 +852,16 @@
         <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I13" s="16" t="str">
-        <x:v>Text-quality analysis</x:v>
+        <x:v>Question-text ambiguity analysis</x:v>
       </x:c>
       <x:c r="J13" s="16" t="str">
-        <x:v>Question text is unreadable</x:v>
+        <x:v>Question text is missing or unreadable</x:v>
       </x:c>
       <x:c r="K13" s="16" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="L13" s="22" t="str">
-        <x:v>Only material ambiguity is evaluated.</x:v>
+        <x:v>A clear reference to an unavailable supporting item is not, by itself, wording ambiguity.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
@@ -877,7 +878,7 @@
         <x:v>Complete Information</x:v>
       </x:c>
       <x:c r="E14" s="16" t="str">
-        <x:v>Each question should contain the information necessary to produce the expected answer.</x:v>
+        <x:v>Each question, together with its confirmed question-specific context, should contain the data, conditions, and supporting material necessary to produce the expected answer.</x:v>
       </x:c>
       <x:c r="F14" s="16" t="str">
         <x:v>Derived Exam Requirement</x:v>
@@ -889,16 +890,16 @@
         <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I14" s="16" t="str">
-        <x:v>Content-completeness analysis</x:v>
+        <x:v>Question and confirmed supporting-context completeness analysis</x:v>
       </x:c>
       <x:c r="J14" s="16" t="str">
-        <x:v>Question or surrounding context is unreadable</x:v>
+        <x:v>Question text or required confirmed context is unreadable or cannot be associated reliably</x:v>
       </x:c>
       <x:c r="K14" s="16" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="L14" s="22" t="str">
-        <x:v>The system does not assess answer-key correctness.</x:v>
+        <x:v>Includes confirmed tables, figures, code, labels, captions, and explicit references; general exam instructions are evaluated separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
@@ -1181,7 +1182,7 @@
         <x:v>Complete Instructions</x:v>
       </x:c>
       <x:c r="E22" s="16" t="str">
-        <x:v>The exam should include necessary general and question-specific instructions.</x:v>
+        <x:v>The exam should include necessary exam-level general instructions.</x:v>
       </x:c>
       <x:c r="F22" s="16" t="str">
         <x:v>Derived Exam Requirement</x:v>
@@ -1193,16 +1194,16 @@
         <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I22" s="16" t="str">
-        <x:v>Instruction analysis</x:v>
+        <x:v>Exam-level instruction analysis</x:v>
       </x:c>
       <x:c r="J22" s="16" t="str">
-        <x:v>Instructions are unreadable</x:v>
+        <x:v>Exam-level instruction text is unreadable</x:v>
       </x:c>
       <x:c r="K22" s="16" t="str">
-        <x:v>No special instruction is needed</x:v>
+        <x:v>No additional exam-level instruction is needed</x:v>
       </x:c>
       <x:c r="L22" s="22" t="str">
-        <x:v>The system does not invent local exam policies.</x:v>
+        <x:v>Limited to general answer requirements, resources or tools, constraints, and submission or formatting directions; question completeness and material availability are evaluated separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
@@ -1550,7 +1551,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd5b2cd2d3b74564"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5aeb1a90b00e4915"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Save reference before auto draft and PDF copy-paste workflow
</commit_message>
<xml_diff>
--- a/knowledge_base/source/04_requirements.xlsx
+++ b/knowledge_base/source/04_requirements.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_requirements" sheetId="1" r:id="R194e9f36926941a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_requirements" sheetId="1" r:id="R556617bc92f44355"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -116,7 +116,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="26">
+  <x:cellXfs count="27">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -179,6 +179,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -801,7 +802,7 @@
         <x:v>Clear Task Statement</x:v>
       </x:c>
       <x:c r="E12" s="16" t="str">
-        <x:v>Each question should state a clear task and recognizable response expectation.</x:v>
+        <x:v>Each question should state a recognizable action and the response or output expected from the student.</x:v>
       </x:c>
       <x:c r="F12" s="16" t="str">
         <x:v>Derived Exam Requirement</x:v>
@@ -813,16 +814,16 @@
         <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I12" s="16" t="str">
-        <x:v>Text-quality analysis</x:v>
+        <x:v>Question-text task analysis</x:v>
       </x:c>
       <x:c r="J12" s="16" t="str">
-        <x:v>OCR confidence is insufficient</x:v>
+        <x:v>Question text is unreadable or OCR confidence is insufficient</x:v>
       </x:c>
       <x:c r="K12" s="16" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="L12" s="22" t="str">
-        <x:v>Style preferences alone are not evaluated.</x:v>
+        <x:v>Limited to the task action and expected response; supporting-material availability, information completeness, and exam-level instructions are evaluated separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
@@ -839,7 +840,7 @@
         <x:v>Unambiguous Wording</x:v>
       </x:c>
       <x:c r="E13" s="16" t="str">
-        <x:v>Question wording should avoid ambiguity, contradiction, or missing conditions that materially affect interpretation.</x:v>
+        <x:v>Question wording should avoid linguistic ambiguity, contradiction, unclear terminology, or wording that materially permits different interpretations.</x:v>
       </x:c>
       <x:c r="F13" s="16" t="str">
         <x:v>Derived Exam Requirement</x:v>
@@ -851,16 +852,16 @@
         <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I13" s="16" t="str">
-        <x:v>Text-quality analysis</x:v>
+        <x:v>Question-text ambiguity analysis</x:v>
       </x:c>
       <x:c r="J13" s="16" t="str">
-        <x:v>Question text is unreadable</x:v>
+        <x:v>Question text is missing or unreadable</x:v>
       </x:c>
       <x:c r="K13" s="16" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="L13" s="22" t="str">
-        <x:v>Only material ambiguity is evaluated.</x:v>
+        <x:v>A clear reference to an unavailable supporting item is not, by itself, wording ambiguity.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
@@ -877,7 +878,7 @@
         <x:v>Complete Information</x:v>
       </x:c>
       <x:c r="E14" s="16" t="str">
-        <x:v>Each question should contain the information necessary to produce the expected answer.</x:v>
+        <x:v>Each question, together with its confirmed question-specific context, should contain the data, conditions, and supporting material necessary to produce the expected answer.</x:v>
       </x:c>
       <x:c r="F14" s="16" t="str">
         <x:v>Derived Exam Requirement</x:v>
@@ -889,16 +890,16 @@
         <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I14" s="16" t="str">
-        <x:v>Content-completeness analysis</x:v>
+        <x:v>Question and confirmed supporting-context completeness analysis</x:v>
       </x:c>
       <x:c r="J14" s="16" t="str">
-        <x:v>Question or surrounding context is unreadable</x:v>
+        <x:v>Question text or required confirmed context is unreadable or cannot be associated reliably</x:v>
       </x:c>
       <x:c r="K14" s="16" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="L14" s="22" t="str">
-        <x:v>The system does not assess answer-key correctness.</x:v>
+        <x:v>Includes confirmed tables, figures, code, labels, captions, and explicit references; general exam instructions are evaluated separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
@@ -1181,7 +1182,7 @@
         <x:v>Complete Instructions</x:v>
       </x:c>
       <x:c r="E22" s="16" t="str">
-        <x:v>The exam should include necessary general and question-specific instructions.</x:v>
+        <x:v>The exam should include necessary exam-level general instructions.</x:v>
       </x:c>
       <x:c r="F22" s="16" t="str">
         <x:v>Derived Exam Requirement</x:v>
@@ -1193,16 +1194,16 @@
         <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I22" s="16" t="str">
-        <x:v>Instruction analysis</x:v>
+        <x:v>Exam-level instruction analysis</x:v>
       </x:c>
       <x:c r="J22" s="16" t="str">
-        <x:v>Instructions are unreadable</x:v>
+        <x:v>Exam-level instruction text is unreadable</x:v>
       </x:c>
       <x:c r="K22" s="16" t="str">
-        <x:v>No special instruction is needed</x:v>
+        <x:v>No additional exam-level instruction is needed</x:v>
       </x:c>
       <x:c r="L22" s="22" t="str">
-        <x:v>The system does not invent local exam policies.</x:v>
+        <x:v>Limited to general answer requirements, resources or tools, constraints, and submission or formatting directions; question completeness and material availability are evaluated separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
@@ -1550,7 +1551,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd5b2cd2d3b74564"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5aeb1a90b00e4915"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Final pre-deployment version - preserve GitHub history
</commit_message>
<xml_diff>
--- a/knowledge_base/source/04_requirements.xlsx
+++ b/knowledge_base/source/04_requirements.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_requirements" sheetId="1" r:id="R194e9f36926941a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_requirements" sheetId="1" r:id="R556617bc92f44355"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -116,7 +116,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="26">
+  <x:cellXfs count="27">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -179,6 +179,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -801,7 +802,7 @@
         <x:v>Clear Task Statement</x:v>
       </x:c>
       <x:c r="E12" s="16" t="str">
-        <x:v>Each question should state a clear task and recognizable response expectation.</x:v>
+        <x:v>Each question should state a recognizable action and the response or output expected from the student.</x:v>
       </x:c>
       <x:c r="F12" s="16" t="str">
         <x:v>Derived Exam Requirement</x:v>
@@ -813,16 +814,16 @@
         <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I12" s="16" t="str">
-        <x:v>Text-quality analysis</x:v>
+        <x:v>Question-text task analysis</x:v>
       </x:c>
       <x:c r="J12" s="16" t="str">
-        <x:v>OCR confidence is insufficient</x:v>
+        <x:v>Question text is unreadable or OCR confidence is insufficient</x:v>
       </x:c>
       <x:c r="K12" s="16" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="L12" s="22" t="str">
-        <x:v>Style preferences alone are not evaluated.</x:v>
+        <x:v>Limited to the task action and expected response; supporting-material availability, information completeness, and exam-level instructions are evaluated separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
@@ -839,7 +840,7 @@
         <x:v>Unambiguous Wording</x:v>
       </x:c>
       <x:c r="E13" s="16" t="str">
-        <x:v>Question wording should avoid ambiguity, contradiction, or missing conditions that materially affect interpretation.</x:v>
+        <x:v>Question wording should avoid linguistic ambiguity, contradiction, unclear terminology, or wording that materially permits different interpretations.</x:v>
       </x:c>
       <x:c r="F13" s="16" t="str">
         <x:v>Derived Exam Requirement</x:v>
@@ -851,16 +852,16 @@
         <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I13" s="16" t="str">
-        <x:v>Text-quality analysis</x:v>
+        <x:v>Question-text ambiguity analysis</x:v>
       </x:c>
       <x:c r="J13" s="16" t="str">
-        <x:v>Question text is unreadable</x:v>
+        <x:v>Question text is missing or unreadable</x:v>
       </x:c>
       <x:c r="K13" s="16" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="L13" s="22" t="str">
-        <x:v>Only material ambiguity is evaluated.</x:v>
+        <x:v>A clear reference to an unavailable supporting item is not, by itself, wording ambiguity.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
@@ -877,7 +878,7 @@
         <x:v>Complete Information</x:v>
       </x:c>
       <x:c r="E14" s="16" t="str">
-        <x:v>Each question should contain the information necessary to produce the expected answer.</x:v>
+        <x:v>Each question, together with its confirmed question-specific context, should contain the data, conditions, and supporting material necessary to produce the expected answer.</x:v>
       </x:c>
       <x:c r="F14" s="16" t="str">
         <x:v>Derived Exam Requirement</x:v>
@@ -889,16 +890,16 @@
         <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I14" s="16" t="str">
-        <x:v>Content-completeness analysis</x:v>
+        <x:v>Question and confirmed supporting-context completeness analysis</x:v>
       </x:c>
       <x:c r="J14" s="16" t="str">
-        <x:v>Question or surrounding context is unreadable</x:v>
+        <x:v>Question text or required confirmed context is unreadable or cannot be associated reliably</x:v>
       </x:c>
       <x:c r="K14" s="16" t="str">
         <x:v>None</x:v>
       </x:c>
       <x:c r="L14" s="22" t="str">
-        <x:v>The system does not assess answer-key correctness.</x:v>
+        <x:v>Includes confirmed tables, figures, code, labels, captions, and explicit references; general exam instructions are evaluated separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
@@ -1181,7 +1182,7 @@
         <x:v>Complete Instructions</x:v>
       </x:c>
       <x:c r="E22" s="16" t="str">
-        <x:v>The exam should include necessary general and question-specific instructions.</x:v>
+        <x:v>The exam should include necessary exam-level general instructions.</x:v>
       </x:c>
       <x:c r="F22" s="16" t="str">
         <x:v>Derived Exam Requirement</x:v>
@@ -1193,16 +1194,16 @@
         <x:v>Exam evidence only</x:v>
       </x:c>
       <x:c r="I22" s="16" t="str">
-        <x:v>Instruction analysis</x:v>
+        <x:v>Exam-level instruction analysis</x:v>
       </x:c>
       <x:c r="J22" s="16" t="str">
-        <x:v>Instructions are unreadable</x:v>
+        <x:v>Exam-level instruction text is unreadable</x:v>
       </x:c>
       <x:c r="K22" s="16" t="str">
-        <x:v>No special instruction is needed</x:v>
+        <x:v>No additional exam-level instruction is needed</x:v>
       </x:c>
       <x:c r="L22" s="22" t="str">
-        <x:v>The system does not invent local exam policies.</x:v>
+        <x:v>Limited to general answer requirements, resources or tools, constraints, and submission or formatting directions; question completeness and material availability are evaluated separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
@@ -1550,7 +1551,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd5b2cd2d3b74564"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5aeb1a90b00e4915"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>